<commit_message>
fix: homepage critique fixes for desktop and mobile parity
- Proxima Nova weight mapping matching alc.ca (bold renders semibold)
- mobile-only 'Check winning numbers' banner section
- mobile image crops for hero carousel and right-rail promos
- jackpot strip '+ 90' and est. styling, header utility alignment, footer mobile spacing

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,10 +73,13 @@
     <t>index.report.json</t>
   </si>
   <si>
+    <t>["carousel-promo","carousel-winners","cards-game","cards-promo","cards-promo"]</t>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
-    <t>2026-10-15T03:10:36.647Z</t>
+    <t>2026-10-16T11:54:49.687Z</t>
   </si>
   <si>
     <t>content/alc/en.html.report.json</t>
@@ -570,7 +573,7 @@
         <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
         <v>12</v>
@@ -579,7 +582,7 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -588,7 +591,7 @@
         <v>15</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s">
         <v>17</v>
@@ -599,28 +602,28 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
         <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I4" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
feat: online game detail template (casino, instant-win, live casino)
- new blocks: hero-game, carousel-thumbnails, tabs-boxed; cards-game rail variant
- auto breadcrumbs from page metadata, game-detail main/rail section layout
- import script, parsers and transformer rules for 731 game pages; lowercase link paths,
  alc.ca-hosted assets and game launchers linked absolutely, og:title for slug titles

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="46">
   <si>
     <t>_reportFile</t>
   </si>
@@ -79,7 +79,7 @@
     <t>index</t>
   </si>
   <si>
-    <t>2026-10-16T11:54:49.687Z</t>
+    <t>2026-10-16T15:15:06.674Z</t>
   </si>
   <si>
     <t>content/alc/en.html.report.json</t>
@@ -104,6 +104,57 @@
   </si>
   <si>
     <t>2026-10-15T03:09:28.474Z</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/10000-wolves-10k-ways.report.json</t>
+  </si>
+  <si>
+    <t>["hero-game","carousel-thumbnails","tabs-boxed","cards-game"]</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/10000-wolves-10k-ways</t>
+  </si>
+  <si>
+    <t>online-game-detail</t>
+  </si>
+  <si>
+    <t>2026-10-16T15:14:18.601Z</t>
+  </si>
+  <si>
+    <t>10000-wolves-10k-ways</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/10000-wolves-10k-ways.html</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/ultimate-texas-holdem-live.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/casino/ultimate-texas-holdem-live</t>
+  </si>
+  <si>
+    <t>2026-10-16T15:14:39.982Z</t>
+  </si>
+  <si>
+    <t>ultimate-texas-holdem-live</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/casino/ultimate-texas-holdem-live.html</t>
+  </si>
+  <si>
+    <t>en/play-online/instant-win-games/zombieville.report.json</t>
+  </si>
+  <si>
+    <t>en/play-online/instant-win-games/zombieville</t>
+  </si>
+  <si>
+    <t>2026-10-16T15:14:30.072Z</t>
+  </si>
+  <si>
+    <t>zombieville</t>
+  </si>
+  <si>
+    <t>https://www.alc.ca/content/alc/en/play-online/instant-win-games/zombieville.html</t>
   </si>
 </sst>
 </file>
@@ -492,16 +543,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="33" customWidth="1"/>
-    <col min="2" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="21" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="1" max="5" width="50" customWidth="1"/>
+    <col min="7" max="7" width="20" customWidth="1"/>
     <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="50" customWidth="1"/>
-    <col min="10" max="10" width="40" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -630,6 +678,102 @@
       </c>
       <c r="J4" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" t="s">
+        <v>33</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J7" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>